<commit_message>
Verificar MySQL local y cerrar evidencias del capítulo V
</commit_message>
<xml_diff>
--- a/docs/Matriz_Pruebas_Integrador_II_Verificada.xlsx
+++ b/docs/Matriz_Pruebas_Integrador_II_Verificada.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GRUPO 2" sheetId="1" r:id="R08f549f86b394e4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GRUPO 2" sheetId="1" r:id="R4da5f73ae8684cf9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -510,19 +510,19 @@
         <x:v>Listado, búsqueda y filtro de productos</x:v>
       </x:c>
       <x:c r="F6" s="5" t="str">
-        <x:v>API local perfil demo H2 con 4 productos</x:v>
+        <x:v>API local conectada a MySQL 8.4 con 20 productos; capturas de interfaz obtenidas antes en H2.</x:v>
       </x:c>
       <x:c r="G6" s="5" t="str">
-        <x:v>Abrir catalogo.html sin ?demo=1; buscar paracetamol en el campo del catálogo.</x:v>
+        <x:v>Consultar GET /api/productos con MySQL; revisar el catálogo y la búsqueda en las capturas de interfaz.</x:v>
       </x:c>
       <x:c r="H6" s="5" t="str">
         <x:v>La lista se reduce a los productos coincidentes y muestra precio y stock del backend.</x:v>
       </x:c>
       <x:c r="I6" s="5" t="str">
-        <x:v>Observación local en Firefox; GET /api/productos; ApiFlowTests.java</x:v>
+        <x:v>docs/evidencias/verificacion_mysql.json; docs/evidencias/01_catalogo_h2.png y 02_busqueda_h2.png.</x:v>
       </x:c>
       <x:c r="J6" s="5" t="str">
-        <x:v>4 productos cargados; al buscar paracetamol apareció 1 producto con stock 24 y precio S/ 12.90. Falta repetir con MySQL y catálogo completo.</x:v>
+        <x:v>La API MySQL devolvió 20 productos. La visualización y búsqueda fueron observadas en H2; falta repetir esa interacción de interfaz con MySQL.</x:v>
       </x:c>
       <x:c r="K6" s="5" t="str">
         <x:v>Parcial</x:v>
@@ -542,22 +542,22 @@
         <x:v>Crear orden con detalle y descontar stock</x:v>
       </x:c>
       <x:c r="F7" s="4" t="str">
-        <x:v>Cliente autenticado; producto sin receta, stock 3</x:v>
+        <x:v>API local conectada a MySQL 8.4; producto de prueba con stock inicial de 24 unidades.</x:v>
       </x:c>
       <x:c r="G7" s="4" t="str">
-        <x:v>Ejecutar catalogAndCheckoutUseServerPriceAndUpdateStockAtomically; solicitar 2 unidades con total manipulado.</x:v>
+        <x:v>Registrar cliente de prueba, enviar pedido sin receta por API, consultar historial y comprobar pedido, detalle y stock en MySQL tras reiniciar Spring Boot.</x:v>
       </x:c>
       <x:c r="H7" s="4" t="str">
         <x:v>El servidor calcula el total, crea ORD, guarda detalle, reduce stock y rechaza otra compra si no alcanza.</x:v>
       </x:c>
       <x:c r="I7" s="4" t="str">
-        <x:v>backend/src/test/java/com/merysalud/ApiFlowTests.java</x:v>
+        <x:v>docs/evidencias/verificacion_mysql.json; backend/src/test/java (pruebas automatizadas en H2).</x:v>
       </x:c>
       <x:c r="J7" s="4" t="str">
-        <x:v>Prueba automática aprobada: total S/ 30.80, stock de 3 a 1, detalle persistido; segunda petición devuelve 409. Pago y WhatsApp no son parte de esta prueba.</x:v>
+        <x:v>Pedido ORD-5F0CF7B3-FF0 persistido con un detalle; stock 24→23; aparece en historial del cliente y se conserva después del reinicio. Interfaz de compra observada previamente en H2.</x:v>
       </x:c>
       <x:c r="K7" s="4" t="str">
-        <x:v>Aceptado en H2</x:v>
+        <x:v>Aceptado API/MySQL</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="257.25" hidden="0" customHeight="1">
@@ -574,22 +574,22 @@
         <x:v>Tiempo de GET /api/productos</x:v>
       </x:c>
       <x:c r="F8" s="5" t="str">
-        <x:v>Backend local perfil demo H2, 4 productos</x:v>
+        <x:v>Backend local conectado a MySQL 8.4; catálogo de 20 productos; 3 solicitudes de calentamiento.</x:v>
       </x:c>
       <x:c r="G8" s="5" t="str">
-        <x:v>Enviar 30 solicitudes secuenciales al endpoint; registrar min, mediana, p95 y máximo.</x:v>
+        <x:v>Ejecutar 30 consultas secuenciales GET /api/productos y registrar mínimo, mediana, percentil 95 y máximo.</x:v>
       </x:c>
       <x:c r="H8" s="5" t="str">
         <x:v>Cada respuesta no supera 3000 ms en el entorno medido.</x:v>
       </x:c>
       <x:c r="I8" s="5" t="str">
-        <x:v>docs/evidencias/medicion_catalogo_h2.json</x:v>
+        <x:v>scripts/medir-catalogo.py; docs/evidencias/medicion_catalogo_mysql.json.</x:v>
       </x:c>
       <x:c r="J8" s="5" t="str">
-        <x:v>30 muestras: mínimo 2.30 ms, mediana 3.42 ms, p95 6.01 ms, máximo 6.23 ms. Falta medición con MySQL, catálogo completo y equipo de entrega.</x:v>
+        <x:v>30 muestras: mínimo 2,53 ms; mediana 3,81 ms; p95 6,23 ms; máximo 6,44 ms. Cumple 3000 ms solo en este equipo local; no es prueba concurrente.</x:v>
       </x:c>
       <x:c r="K8" s="5" t="str">
-        <x:v>Parcial</x:v>
+        <x:v>Aceptado local</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="257.25" hidden="0" customHeight="1">

</xml_diff>